<commit_message>
Add solution for Key Races problem (LeetCode 835A)
- Implemented a C++ program to determine the winner between two racers based on their speeds and time penalties.
- The program reads input values for distance, speeds, and penalties, then calculates the total time for each racer and outputs the result.
</commit_message>
<xml_diff>
--- a/LeetCode/Top Leetcode questions of All Time - most important.xlsx
+++ b/LeetCode/Top Leetcode questions of All Time - most important.xlsx
@@ -2462,7 +2462,6 @@
   <fonts count="16">
     <font>
       <sz val="11.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -2480,13 +2479,11 @@
     <font>
       <b/>
       <sz val="20.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="24.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -2515,7 +2512,6 @@
     <font>
       <u/>
       <sz val="11.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -2527,18 +2523,15 @@
     <font>
       <b/>
       <sz val="18.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
       <sz val="12.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="12.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -2570,7 +2563,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="64"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -2617,14 +2609,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
+  <borders count="1">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -2641,61 +2626,61 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="1" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="1" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="2" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="3" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="3" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="4" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="4" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="4" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="4" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="0" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="5" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="5" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="5" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="5" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="5" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="5" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="1" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
@@ -2705,90 +2690,90 @@
     <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="7" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="7" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="7" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="7" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="5" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="5" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="5" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="5" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="0" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="5" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="5" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="5" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="8" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="5" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="8" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="8" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="8" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="5" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="5" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="5" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="8" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="5" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="8" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="8" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="8" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf fontId="9" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="8" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="8" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="8" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="8" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf fontId="10" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="10" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="10" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="10" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="11" fillId="9" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="11" fillId="9" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="11" fillId="9" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="11" fillId="9" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf fontId="6" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="6" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="0" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf fontId="0" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="6" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="6" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="5" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="11" fillId="9" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="11" fillId="9" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf fontId="12" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
@@ -2798,33 +2783,33 @@
     <xf fontId="12" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="10" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="13" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="13" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="13" fillId="10" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="13" fillId="10" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="12" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="14" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="12" fillId="10" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="14" fillId="10" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="12" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="12" fillId="10" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="13" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="13" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="13" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="13" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="12" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="12" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="14" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="12" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="14" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="14" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="12" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="14" fillId="8" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="15" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="15" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3560,7 +3545,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>9</v>

</xml_diff>